<commit_message>
Date de contact Pepiniera Doi Cocoși (telefon, adresă) în comenzi, cererea de ofertă și lista de oferte
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/comenzi-miyawaki-est.xlsx
+++ b/resurse/oferte/comenzi-miyawaki-est.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>apare în lista pepinierelor silvice cu prețuri neintroduse (0,01 lei) · de sunat pentru preț și stoc real</t>
+          <t>tel. 0766405638 · strada Doi Cocoși nr. 2, Brăila · apare în lista pepinierelor silvice cu prețuri neintroduse (0,01 lei) · de sunat pentru preț și stoc real</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>apare în lista pepinierelor silvice cu prețuri neintroduse (0,01 lei) · de sunat pentru preț și stoc real</t>
+          <t>tel. 0766405638 · strada Doi Cocoși nr. 2, Brăila · apare în lista pepinierelor silvice cu prețuri neintroduse (0,01 lei) · de sunat pentru preț și stoc real</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stocul Pepinierei Silvice Agigea (telefon, 21 octombrie 2026)
- comenzi-miyawaki-est: Agigea confirmă porumbar și scumpie (plus măceș,
  jugastru, stejar brumăriu, cer, corcoduș, vișin turcesc, păducel, sălcioară);
  nu are corn, alun, salbă, călin, dârmox, pin negru, soc, arbore de mazăre,
  sorb, păr sălbatic, arțar tătăresc, sâmbovină → secțiune nouă „Specii încă
  fără furnizor”, stare și ordinea apelurilor actualizate (Salcea urmează)
- fișa furnizorilor, comenzile planului nord (sălcioară) și jurnalul

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/comenzi-miyawaki-est.xlsx
+++ b/resurse/oferte/comenzi-miyawaki-est.xlsx
@@ -13,9 +13,10 @@
     <sheet name="Pepiniera Doi Cocoși SRL" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Pepiniera Țuțora" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Pepiniera Silvică Agigea" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Pepiniera Selficom" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Pepiniera Cobadin" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Pepiniera Mizil" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Specii încă fără furnizor" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Pepiniera Selficom" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Pepiniera Cobadin" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Pepiniera Mizil" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -602,13 +603,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>290</v>
+        <v>85</v>
       </c>
       <c r="D7" t="n">
-        <v>324</v>
+        <v>94</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -617,169 +618,180 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DN 38, Agigea · tel. 0241738043, 0748143025 (ing. Orac) · pepiniera@constanta.rosilva.ro · ofertă pe bursataraneasca.ro: porumbar 0,50 lei/buc fără TVA, valabilă 30 septembrie – 14 octombrie 2026 · 70 km de Crucea</t>
+          <t>DN 38, Agigea · tel. 0241738043, 0748143025 (ing. Orac) · pepiniera@constanta.rosilva.ro · 70 km de Crucea · stoc confirmat telefonic la 21 octombrie 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pepiniera Selficom — Galați</t>
+          <t>Specii încă fără furnizor — după răspunsul de la Agigea (21 octombrie 2026)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>33</v>
+        <v>205</v>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
-      </c>
-      <c r="E8" t="n">
-        <v>44</v>
+        <v>230</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>la cerere</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
+          <t>nicio pepinieră confirmată; următoarele apeluri: Salcea (Romsilva Suceava), Tomești (Harghita), ICAS Ștefănești, Voivodeni (Reghin), OLMA Iași, online</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pepiniera Cobadin — Constanța</t>
+          <t>Pepiniera Selficom — Galați</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>la cerere</t>
-        </is>
+        <v>37</v>
+      </c>
+      <c r="E9" t="n">
+        <v>44</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
+          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Pepiniera Cobadin — Constanța</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>22</v>
+      </c>
+      <c r="D10" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>la cerere</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Pepiniera Mizil — Prahova (magazin online)</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>4</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C11" t="n">
         <v>125</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>139</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E11" t="n">
         <v>2142</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>www.pepinieramizil.ro · livrare prin curier, transport gratuit peste 500 lei · prețurile se verifică pe site la comandă</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C12" s="3" t="n">
         <v>919</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D12" s="3" t="n">
         <v>1025</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E12" s="3" t="n">
         <v>2671</v>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>plus Cobadin și Mizil la cerere; total orientativ 3 000–5 500 lei</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Înlocuiri (speciile care nu se găsesc)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Specie din schemă</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>În schemă</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Înlocuitor și furnizor</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Cărpiniță (Carpinus orientalis)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>38</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>19 carpen comun (Țuțora Iași) + 19 sâmbovină (Agigea, de întrebat; Cobadin 50 lei; altfel tot carpen)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Salbă râioasă (Euonymus verrucosus)</t>
+          <t>Cărpiniță (Carpinus orientalis)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>27 salbă moale (Mizil, 9,91 lei)</t>
+          <t>19 carpen comun (Țuțora Iași) + 19 sâmbovină (Agigea nu are; Cobadin 50 lei; altfel tot carpen)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Verigar (Rhamnus cathartica)</t>
+          <t>Salbă râioasă (Euonymus verrucosus)</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -787,29 +799,29 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16 călin (Mizil, 18,02 lei) + 11 măceș (Foresta)</t>
+          <t>27 salbă moale (Mizil, 9,91 lei)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Iasomie sălbatică (Jasminum fruticans)</t>
+          <t>Verigar (Rhamnus cathartica)</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>22 cătină roșie, Tamarix (Cobadin, 15 lei)</t>
+          <t>16 călin (Mizil, 18,02 lei) + 11 măceș (Foresta)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bășicoasă (Colutea arborescens)</t>
+          <t>Iasomie sălbatică (Jasminum fruticans)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -817,9 +829,254 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>22 arbore de mazăre, Caragana (Agigea, de întrebat; Mizil nu are stoc)</t>
-        </is>
-      </c>
+          <t>22 cătină roșie, Tamarix (Cobadin, 15 lei)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Bășicoasă (Colutea arborescens)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>22</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>22 arbore de mazăre, Caragana (Agigea nu are; Mizil fără stoc; de găsit sau înlocuit cu păducel)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Pepiniera Mizil — Prahova (magazin online)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>www.pepinieramizil.ro · livrare prin curier, transport gratuit peste 500 lei · prețurile se verifică pe site la comandă</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>**Oferta primită la 6 octombrie** (`raspunsuri/oferta-pepiniera-mizil-2026-10.xlsx`): au doar 4 din cele 12 specii cerute: corn 18,90 lei, alun 13,51 lei, salbă moale 9,91 lei, călin 18,02 lei. Lipsesc sorb, păr sălbatic, cireș sălbatic, porumbar, dârmox, soc, arbore de mazăre și pin negru, mutate la Agigea și Doi Cocoși. Prețurile sunt de 10–15 ori peste pepinierele silvice, deci cornul și alunul se întreabă întâi la Agigea; dacă nu le au, rămân aici. Se cer mărimile cele mai mici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cod schemă</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Specie de comandat</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nume latin</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>În schemă</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>De comandat (+10 %)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Preț (lei/buc)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Observații</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Cm</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Corn</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Cornus mas</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>18,90</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>strat C; Agigea nu are (21 octombrie); înainte de Mizil se încearcă Tomești (Harghita) și ICAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Alun</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Corylus avellana</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>13,51</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>strat C; Agigea nu are (21 octombrie); se încearcă Pepiniera Stejarul, Galați, 0774609287</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Ev</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Salbă moale (în locul salbei râioase)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Euonymus europaeus</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>9,91</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>strat D; înlocuitor; Mizil are</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Rh</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Călin (în locul verigarului)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Viburnum opulus</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>18,02</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>strat D; înlocuitor pentru 16 din cei 27 verigari (restul 11 = măceș, la Foresta); Mizil are</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr"/>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>139</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1719,7 +1976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1741,14 +1998,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DN 38, Agigea · tel. 0241738043, 0748143025 (ing. Orac) · pepiniera@constanta.rosilva.ro · ofertă pe bursataraneasca.ro: porumbar 0,50 lei/buc fără TVA, valabilă 30 septembrie – 14 octombrie 2026 · 70 km de Crucea</t>
+          <t>DN 38, Agigea · tel. 0241738043, 0748143025 (ing. Orac) · pepiniera@constanta.rosilva.ro · 70 km de Crucea · stoc confirmat telefonic la 21 octombrie 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pepiniera silvică de stat a Dobrogei: produce speciile folosite la împăduririle și perdelele din județ, exact lista pădurii. Porumbarul e în ofertă acum, la 0,50 lei; pentru celelalte specii de mai jos se întreabă la telefon, pentru că oferta publicată e scurtă. Tot aici se întreabă și de corn, alun, păducel, lemn câinesc, sălcioară, ca să scadă dependența de Mizil (unde cornul e 18,90 lei și alunul 13,51). De sunat **săptămâna aceasta**: oferta de porumbar expiră pe 14 octombrie.</t>
+          <t>**Răspuns telefonic, 21 octombrie 2026.** Au în stoc: **porumbar, scumpie, măceș, jugastru, stejar brumăriu, cer, corcoduș, vișin turcesc, păducel** (toate în schemă) și **sălcioară** (perdelele planului nord), plus frasin de Pennsylvania, stejar verde (*Quercus ilex*), ienupăr de Virginia, glădiță și varietăți de plop, care nu intră în proiect (frasinul de Pennsylvania și glădița sunt invazive, stejarul verde nu rezistă la gerurile din Crucea, plopul nu are loc). **Nu au**: corn, alun, salbă moale, călin, dârmox, pin negru, soc, arbore de mazăre, sorb, păr sălbatic, arțar tătăresc, sâmbovină. Prețurile și mărimile nu au fost discutate; se cer la comanda fermă. De la ei se iau sigur porumbarul și scumpia; jugastrul (acum la Doi Cocoși, preț neconfirmat) și speciile comune cu Foresta (stejar brumăriu, cer, corcoduș, vișin turcesc, păducel, măceș) se pot muta aici dacă prețul e la fel, ca să scadă un transport: Agigea e la 70 km, Brăila la 150.</t>
         </is>
       </c>
     </row>
@@ -1818,31 +2075,31 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>strat D, manta ghimpoasă; ofertă publicată, mii de bucăți; alternativ planteieftine.ro 5,40 lei (30–50 cm, rădăcină liberă)</t>
+          <t>strat D, manta ghimpoasă; în stoc (21 octombrie); prețul din oferta de pe bursataraneasca.ro, de reconfirmat</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Pn</t>
+          <t>Cc</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Pin negru</t>
+          <t>Scumpie</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Pinus nigra</t>
+          <t>Cotinus coggygria</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -1851,290 +2108,26 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>strat A; specia de bază a împăduririlor din Dobrogea, probabil în stoc (puieți de 2–3 ani); dacă nu: Pepiniera Silvică Voivodeni, Reghin, 1,45 lei (transport lung) sau ghiveci de 2–3 l la 45–60 lei online</t>
+          <t>strat C; în stoc (21 octombrie); Cobadin 80 lei era prea scump, Mizil nu mai e nevoie</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Sn</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Soc</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Sambucus nigra</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>strat D; alternativ planteieftine.ro 5 lei (50–80 cm, rădăcină liberă, în stoc)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Vl</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Dârmox</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Viburnum lantana</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>44</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>49</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>strat D; specie de perdea în Dobrogea; alternativ Pepiniera Silvică Salcea, Suceava, 0751164370 (apare în lista lor), sau GardenExpert 21,80 lei; Mizil 30–44 lei, fără stoc acum</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Arbore de mazăre (în locul bășicoasei)</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Caragana arborescens</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>strat D; folosit în perdelele din Dobrogea; Mizil fără stoc; alternativ Pepiniera Roșie 35 lei (scump) sau înlocuire cu 22 păducel de la Foresta</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>St</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Sorb</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Sorbus torminalis</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>strat A; greu de găsit: Mizil 13–15 lei fără stoc, 2biz.ro; dacă nu există nicăieri, se înlocuiește cu 11 cer de la Foresta (strat A) și pădurea rămâne cu 29 de specii</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Pp</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Păr sălbatic</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Pyrus pyraster</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>strat B; alternativ SC OLMA, Iași, 0767806245, 2,5 lei</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>At</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Arțar tătăresc</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Acer tataricum</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>strat B; specie de perdea în Dobrogea; Cobadin are doar exemplare de 6 ani la 100 lei; alternativ Mizil (listat pe site, preț la cerere)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Cc</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Scumpie</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Cotinus coggygria</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>strat C; folosită la împăduriri pe terenuri degradate în Dobrogea; Cobadin 80 lei (prea scump); alternativ Mizil</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Co</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Sâmbovină (în locul cărpiniței)</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Celtis australis</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>de întrebat</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>strat B; înlocuitor pentru 19 din cele 38 cărpinițe; Cobadin 50 lei (3 ani, 1,5–2,5 m); dacă nu există ieftin, în locul ei tot carpen de la Țuțora</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr"/>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr"/>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr"/>
-      <c r="D16" s="6" t="n">
-        <v>290</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>324</v>
-      </c>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr"/>
+      <c r="C8" s="6" t="inlineStr"/>
+      <c r="D8" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2147,7 +2140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2162,21 +2155,21 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Pepiniera Selficom — Galați</t>
+          <t>Specii încă fără furnizor — după răspunsul de la Agigea (21 octombrie 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
+          <t>nicio pepinieră confirmată; următoarele apeluri: Salcea (Romsilva Suceava), Tomești (Harghita), ICAS Ștefănești, Voivodeni (Reghin), OLMA Iași, online</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Singura pepinieră din zonă cu sânger la preț silvic (Cobadin nu-l are în lista de prețuri). Se ridică odată cu stejarul pufos de la Matto Medusa, sau se cere Agigei.</t>
+          <t>Agigea nu are niciuna dintre speciile de mai jos (nici cornul, alunul, salba moale și călinul, care rămân în secțiunea Mizil ca ultimă variantă). Sursele din coloana „Observații” sunt cele găsite până acum, toate de confirmat telefonic; cantitățile nu intră în costul cunoscut.</t>
         </is>
       </c>
     </row>
@@ -2220,17 +2213,17 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Cs</t>
+          <t>Pn</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Sânger</t>
+          <t>Pin negru</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Cornus sanguinea</t>
+          <t>Pinus nigra</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
@@ -2241,31 +2234,262 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>1,20</t>
+          <t>de găsit</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>strat C; alternativ Pepiniera Zăval (Dolj) 1,02 lei sau Agigea</t>
+          <t>strat A; Pepiniera Silvică Voivodeni, Reghin, 1,45 lei (transport lung); de întrebat și la Salcea; altfel ghiveci de 2–3 l la 45–60 lei online</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr"/>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Vl</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Dârmox</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Viburnum lantana</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>strat D; Pepiniera Silvică Salcea, Suceava, 0751164370 (în lista lor); GardenExpert 21,80 lei</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Sn</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Soc</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Sambucus nigra</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>strat D; planteieftine.ro 5 lei (50–80 cm, rădăcină liberă); de întrebat la Salcea</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Arbore de mazăre (în locul bășicoasei)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Caragana arborescens</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>strat D; Pepiniera Roșie 35 lei (scump); altfel înlocuire cu 22 păducel de la Foresta sau Agigea</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>St</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Sorb</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Sorbus torminalis</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>strat A; 2biz.ro 15 lei, 40–60 cm; de întrebat la Salcea; dacă nu există, se înlocuiește cu cer de la Foresta/Agigea și pădurea rămâne cu 29 de specii</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Pp</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Păr sălbatic</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Pyrus pyraster</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>strat B; SC OLMA, Iași, 0767806245, 2,5 lei; de întrebat la Salcea și Doi Cocoși</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>At</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Arțar tătăresc</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Acer tataricum</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>strat B; Mizil (listat pe site, preț la cerere); Cobadin doar exemplare de 6 ani la 100 lei; de întrebat la Salcea și Foresta</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Sâmbovină (în locul cărpiniței)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Celtis australis</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>strat B; Cobadin 50 lei (3 ani, prea scump); dacă nu se găsește ieftin, tot carpen de la Țuțora, adică 38 carpeni în total</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr"/>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr"/>
-      <c r="D7" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>37</v>
-      </c>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="6" t="n">
+        <v>205</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>230</v>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2293,21 +2517,21 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Pepiniera Cobadin — Constanța</t>
+          <t>Pepiniera Selficom — Galați</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
+          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lista lor de prețuri arată **material de amenajare, nu puieți de împădurire**: arbori de 3–9 ani și 1,5–3,5 m la 50–160 lei, arbuști de 0,5–1,5 m la 15–80 lei; sânger și tei argintiu nu sunt în listă. Pentru pădure rămâne de la ei doar cătina roșie (15 lei, 3 ani, peste 1,3 m, se scurtează la 50 cm la plantare). Arțarul tătăresc, scumpia și sâmbovina s-au mutat la Agigea, cu Mizil ca rezervă; sângerul la Selficom Galați. Cererea de ofertă trimisă rămâne valabilă: dacă au și mărimi mici din semănătură, cum au la salcâm japonez (5 lei), se revine.</t>
+          <t>Singura pepinieră din zonă cu sânger la preț silvic (Cobadin nu-l are în lista de prețuri). Se ridică odată cu stejarul pufos de la Matto Medusa, sau se cere Agigei.</t>
         </is>
       </c>
     </row>
@@ -2351,33 +2575,33 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Jf</t>
+          <t>Cs</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Cătină roșie (în locul iasomiei sălbatice)</t>
+          <t>Sânger</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Tamarix ramosissima</t>
+          <t>Cornus sanguinea</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>15,00 (2024)</t>
+          <t>1,20</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>strat D, manta; înlocuitor pentru iasomia sălbatică; alternativ planteieftine.ro Tamarix tetrandra, rădăcină liberă</t>
+          <t>strat C; alternativ Pepiniera Zăval (Dolj) 1,02 lei sau Agigea</t>
         </is>
       </c>
     </row>
@@ -2390,10 +2614,10 @@
       </c>
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
@@ -2409,7 +2633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2424,21 +2648,21 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Pepiniera Mizil — Prahova (magazin online)</t>
+          <t>Pepiniera Cobadin — Constanța</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>www.pepinieramizil.ro · livrare prin curier, transport gratuit peste 500 lei · prețurile se verifică pe site la comandă</t>
+          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>**Oferta primită la 6 octombrie** (`raspunsuri/oferta-pepiniera-mizil-2026-10.xlsx`): au doar 4 din cele 12 specii cerute: corn 18,90 lei, alun 13,51 lei, salbă moale 9,91 lei, călin 18,02 lei. Lipsesc sorb, păr sălbatic, cireș sălbatic, porumbar, dârmox, soc, arbore de mazăre și pin negru, mutate la Agigea și Doi Cocoși. Prețurile sunt de 10–15 ori peste pepinierele silvice, deci cornul și alunul se întreabă întâi la Agigea; dacă nu le au, rămân aici. Se cer mărimile cele mai mici.</t>
+          <t>Lista lor de prețuri arată **material de amenajare, nu puieți de împădurire**: arbori de 3–9 ani și 1,5–3,5 m la 50–160 lei, arbuști de 0,5–1,5 m la 15–80 lei; sânger și tei argintiu nu sunt în listă. Pentru pădure rămâne de la ei doar cătina roșie (15 lei, 3 ani, peste 1,3 m, se scurtează la 50 cm la plantare). Arțarul tătăresc, scumpia și sâmbovina s-au mutat la Agigea, cu Mizil ca rezervă; sângerul la Selficom Galați. Cererea de ofertă trimisă rămâne valabilă: dacă au și mărimi mici din semănătură, cum au la salcâm japonez (5 lei), se revine.</t>
         </is>
       </c>
     </row>
@@ -2482,151 +2706,52 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Cm</t>
+          <t>Jf</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Corn</t>
+          <t>Cătină roșie (în locul iasomiei sălbatice)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Cornus mas</t>
+          <t>Tamarix ramosissima</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>18,90</t>
+          <t>15,00 (2024)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>strat C; de întrebat întâi la Agigea; Mizil are</t>
+          <t>strat D, manta; înlocuitor pentru iasomia sălbatică; alternativ planteieftine.ro Tamarix tetrandra, rădăcină liberă</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Alun</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Corylus avellana</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>33</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>13,51</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>strat C; alternativ Pepiniera Stejarul, Galați, 0774609287 (preț la cerere) sau Agigea</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Ev</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Salbă moale (în locul salbei râioase)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Euonymus europaeus</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>9,91</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>strat D; înlocuitor; Mizil are</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Rh</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Călin (în locul verigarului)</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Viburnum opulus</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>18,02</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>strat D; înlocuitor pentru 16 din cei 27 verigari (restul 11 = măceș, la Foresta); Mizil are</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr"/>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr"/>
-      <c r="D10" s="6" t="n">
-        <v>125</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>139</v>
-      </c>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Stocul Pepinierei Silvice Salcea (telefon, 21 octombrie 2026)
- Salcea are arțar tătăresc (secțiune nouă, 42 buc prin curier); nu are salbă
  moale, călin, dârmox, sorb, soc, păr sălbatic, pin negru; pinul silvestru
  nu înlocuiește pinul negru
- 11 specii rămân fără furnizor; ordinea apelurilor: Stejarul Galați, Tomești,
  Voivodeni, ICAS, online
- fișa furnizorilor și jurnalul

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/comenzi-miyawaki-est.xlsx
+++ b/resurse/oferte/comenzi-miyawaki-est.xlsx
@@ -13,10 +13,11 @@
     <sheet name="Pepiniera Doi Cocoși SRL" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Pepiniera Țuțora" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Pepiniera Silvică Agigea" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Specii încă fără furnizor" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Pepiniera Selficom" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Pepiniera Cobadin" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Pepiniera Mizil" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pepiniera Silvică Salcea" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Specii încă fără furnizor" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Pepiniera Selficom" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Pepiniera Cobadin" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pepiniera Mizil" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -625,17 +626,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Specii încă fără furnizor — după răspunsul de la Agigea (21 octombrie 2026)</t>
+          <t>Pepiniera Silvică Salcea — Romsilva, Direcția Silvică Suceava</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>205</v>
+        <v>38</v>
       </c>
       <c r="D8" t="n">
-        <v>230</v>
+        <v>42</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -644,169 +645,180 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>nicio pepinieră confirmată; următoarele apeluri: Salcea (Romsilva Suceava), Tomești (Harghita), ICAS Ștefănești, Voivodeni (Reghin), OLMA Iași, online</t>
+          <t>tel. 0753156196 / 0751164370 · stoc confirmat telefonic la 21 octombrie 2026 · livrare prin curier, de stabilit la comandă</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pepiniera Selficom — Galați</t>
+          <t>Specii încă fără furnizor — după răspunsurile de la Agigea și Salcea (21 octombrie 2026)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>33</v>
+        <v>167</v>
       </c>
       <c r="D9" t="n">
-        <v>37</v>
-      </c>
-      <c r="E9" t="n">
-        <v>44</v>
+        <v>188</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>la cerere</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
+          <t>nicio pepinieră confirmată; următoarele apeluri: Stejarul Galați, Tomești (Harghita), Voivodeni (Reghin), ICAS Ștefănești, OLMA Iași, online</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Pepiniera Cobadin — Constanța</t>
+          <t>Pepiniera Selficom — Galați</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D10" t="n">
-        <v>25</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>la cerere</t>
-        </is>
+        <v>37</v>
+      </c>
+      <c r="E10" t="n">
+        <v>44</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
+          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Pepiniera Cobadin — Constanța</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>la cerere</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Pepiniera Mizil — Prahova (magazin online)</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B12" t="n">
         <v>4</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C12" t="n">
         <v>125</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>139</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E12" t="n">
         <v>2142</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>www.pepinieramizil.ro · livrare prin curier, transport gratuit peste 500 lei · prețurile se verifică pe site la comandă</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B13" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C13" s="3" t="n">
         <v>919</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D13" s="3" t="n">
         <v>1025</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E13" s="3" t="n">
         <v>2671</v>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>plus Cobadin și Mizil la cerere; total orientativ 3 000–5 500 lei</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Înlocuiri (speciile care nu se găsesc)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Specie din schemă</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>În schemă</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Înlocuitor și furnizor</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Cărpiniță (Carpinus orientalis)</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>38</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>19 carpen comun (Țuțora Iași) + 19 sâmbovină (Agigea nu are; Cobadin 50 lei; altfel tot carpen)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Salbă râioasă (Euonymus verrucosus)</t>
+          <t>Cărpiniță (Carpinus orientalis)</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>27 salbă moale (Mizil, 9,91 lei)</t>
+          <t>19 carpen comun (Țuțora Iași) + 19 sâmbovină (Agigea nu are; Cobadin 50 lei; altfel tot carpen)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Verigar (Rhamnus cathartica)</t>
+          <t>Salbă râioasă (Euonymus verrucosus)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -814,35 +826,50 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16 călin (Mizil, 18,02 lei) + 11 măceș (Foresta)</t>
+          <t>27 salbă moale (Mizil, 9,91 lei)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Iasomie sălbatică (Jasminum fruticans)</t>
+          <t>Verigar (Rhamnus cathartica)</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>22 cătină roșie, Tamarix (Cobadin, 15 lei)</t>
+          <t>16 călin (Mizil, 18,02 lei) + 11 măceș (Foresta)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bășicoasă (Colutea arborescens)</t>
+          <t>Iasomie sălbatică (Jasminum fruticans)</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>22</v>
       </c>
       <c r="C20" t="inlineStr">
+        <is>
+          <t>22 cătină roșie, Tamarix (Cobadin, 15 lei)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Bășicoasă (Colutea arborescens)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>22</v>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>22 arbore de mazăre, Caragana (Agigea nu are; Mizil fără stoc; de găsit sau înlocuit cu păducel)</t>
         </is>
@@ -854,6 +881,137 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Pepiniera Cobadin — Constanța</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lista lor de prețuri arată **material de amenajare, nu puieți de împădurire**: arbori de 3–9 ani și 1,5–3,5 m la 50–160 lei, arbuști de 0,5–1,5 m la 15–80 lei; sânger și tei argintiu nu sunt în listă. Pentru pădure rămâne de la ei doar cătina roșie (15 lei, 3 ani, peste 1,3 m, se scurtează la 50 cm la plantare). Arțarul tătăresc, scumpia și sâmbovina s-au mutat la Agigea, cu Mizil ca rezervă; sângerul la Selficom Galați. Cererea de ofertă trimisă rămâne valabilă: dacă au și mărimi mici din semănătură, cum au la salcâm japonez (5 lei), se revine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cod schemă</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Specie de comandat</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nume latin</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>În schemă</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>De comandat (+10 %)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Preț (lei/buc)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Observații</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Jf</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Cătină roșie (în locul iasomiei sălbatice)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Tamarix ramosissima</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>15,00 (2024)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>strat D, manta; înlocuitor pentru iasomia sălbatică; alternativ planteieftine.ro Tamarix tetrandra, rădăcină liberă</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2140,368 +2298,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Specii încă fără furnizor — după răspunsul de la Agigea (21 octombrie 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>nicio pepinieră confirmată; următoarele apeluri: Salcea (Romsilva Suceava), Tomești (Harghita), ICAS Ștefănești, Voivodeni (Reghin), OLMA Iași, online</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Agigea nu are niciuna dintre speciile de mai jos (nici cornul, alunul, salba moale și călinul, care rămân în secțiunea Mizil ca ultimă variantă). Sursele din coloana „Observații” sunt cele găsite până acum, toate de confirmat telefonic; cantitățile nu intră în costul cunoscut.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Cod schemă</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Specie de comandat</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Nume latin</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>În schemă</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>De comandat (+10 %)</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Preț (lei/buc)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Observații</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Pn</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Pin negru</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Pinus nigra</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>33</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>strat A; Pepiniera Silvică Voivodeni, Reghin, 1,45 lei (transport lung); de întrebat și la Salcea; altfel ghiveci de 2–3 l la 45–60 lei online</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Vl</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Dârmox</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Viburnum lantana</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>44</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>49</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>strat D; Pepiniera Silvică Salcea, Suceava, 0751164370 (în lista lor); GardenExpert 21,80 lei</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Sn</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Soc</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Sambucus nigra</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>strat D; planteieftine.ro 5 lei (50–80 cm, rădăcină liberă); de întrebat la Salcea</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Arbore de mazăre (în locul bășicoasei)</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Caragana arborescens</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>strat D; Pepiniera Roșie 35 lei (scump); altfel înlocuire cu 22 păducel de la Foresta sau Agigea</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>St</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Sorb</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Sorbus torminalis</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>strat A; 2biz.ro 15 lei, 40–60 cm; de întrebat la Salcea; dacă nu există, se înlocuiește cu cer de la Foresta/Agigea și pădurea rămâne cu 29 de specii</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Pp</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Păr sălbatic</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Pyrus pyraster</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>22</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>strat B; SC OLMA, Iași, 0767806245, 2,5 lei; de întrebat la Salcea și Doi Cocoși</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>At</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Arțar tătăresc</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Acer tataricum</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>strat B; Mizil (listat pe site, preț la cerere); Cobadin doar exemplare de 6 ani la 100 lei; de întrebat la Salcea și Foresta</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Co</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Sâmbovină (în locul cărpiniței)</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Celtis australis</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>19</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>de găsit</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>strat B; Cobadin 50 lei (3 ani, prea scump); dacă nu se găsește ieftin, tot carpen de la Țuțora, adică 38 carpeni în total</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr"/>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr"/>
-      <c r="D14" s="6" t="n">
-        <v>205</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>230</v>
-      </c>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2517,21 +2313,21 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Pepiniera Selficom — Galați</t>
+          <t>Pepiniera Silvică Salcea — Romsilva, Direcția Silvică Suceava</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
+          <t>tel. 0753156196 / 0751164370 · stoc confirmat telefonic la 21 octombrie 2026 · livrare prin curier, de stabilit la comandă</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Singura pepinieră din zonă cu sânger la preț silvic (Cobadin nu-l are în lista de prețuri). Se ridică odată cu stejarul pufos de la Matto Medusa, sau se cere Agigei.</t>
+          <t>**Răspuns telefonic, 21 octombrie 2026.** Au: **arțar tătăresc** (în schemă), pin silvestru, stejar, larice, plop, salcie, salcâm. Nu au salba moale, călinul, dârmoxul și sorbul din lista lor de ornamentale, nici soc, păr sălbatic sau pin negru. Pinul silvestru nu înlocuiește pinul negru: suferă de secetă și arșiță în Dobrogea; rămâne doar ca ultimă variantă. Salcâmul, laricele, plopul, salcia și stejarul pedunculat nu intră în proiect. Prețul și mărimea arțarului, plus costul curierului, se cer la comandă.</t>
         </is>
       </c>
     </row>
@@ -2575,33 +2371,33 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Cs</t>
+          <t>At</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Sânger</t>
+          <t>Arțar tătăresc</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Cornus sanguinea</t>
+          <t>Acer tataricum</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>1,20</t>
+          <t>de întrebat</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>strat C; alternativ Pepiniera Zăval (Dolj) 1,02 lei sau Agigea</t>
+          <t>strat B; în stoc (21 octombrie); singura sursă silvică găsită; livrare prin curier, rădăcină nudă în sac umed</t>
         </is>
       </c>
     </row>
@@ -2614,13 +2410,342 @@
       </c>
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Specii încă fără furnizor — după răspunsurile de la Agigea și Salcea (21 octombrie 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>nicio pepinieră confirmată; următoarele apeluri: Stejarul Galați, Tomești (Harghita), Voivodeni (Reghin), ICAS Ștefănești, OLMA Iași, online</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nici Agigea, nici Salcea nu au speciile de mai jos (nici cornul, alunul, salba moale și călinul, care rămân în secțiunea Mizil ca ultimă variantă). Sursele din coloana „Observații” sunt cele găsite până acum, toate de confirmat telefonic; cantitățile nu intră în costul cunoscut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cod schemă</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Specie de comandat</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nume latin</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>În schemă</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>De comandat (+10 %)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Preț (lei/buc)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Observații</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Pn</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Pin negru</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Pinus nigra</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>strat A; Pepiniera Silvică Voivodeni, Reghin, 1,45 lei (transport lung); Salcea are doar pin silvestru (nepotrivit); altfel ghiveci de 2–3 l la 45–60 lei online</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Vl</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Dârmox</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Viburnum lantana</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>49</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>strat D; Salcea nu are (21 octombrie); de întrebat la Foresta și Doi Cocoși la comanda fermă, la ICAS Ștefănești; GardenExpert 21,80 lei</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Sn</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Soc</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Sambucus nigra</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>strat D; planteieftine.ro 5 lei (50–80 cm, rădăcină liberă); Salcea nu are</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Arbore de mazăre (în locul bășicoasei)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Caragana arborescens</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>strat D; Pepiniera Roșie 35 lei (scump); altfel înlocuire cu 22 păducel de la Foresta sau Agigea</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>St</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Sorb</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Sorbus torminalis</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>strat A; 2biz.ro 15 lei, 40–60 cm; Salcea nu are; dacă nu există, se înlocuiește cu cer de la Foresta/Agigea și pădurea rămâne cu 29 de specii</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Pp</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Păr sălbatic</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Pyrus pyraster</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>strat B; SC OLMA, Iași, 0767806245, 2,5 lei; Salcea nu are; de întrebat la Doi Cocoși</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Sâmbovină (în locul cărpiniței)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Celtis australis</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>de găsit</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>strat B; Cobadin 50 lei (3 ani, prea scump); dacă nu se găsește ieftin, tot carpen de la Țuțora, adică 38 carpeni în total</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr"/>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr"/>
+      <c r="D13" s="6" t="n">
+        <v>167</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>188</v>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2648,21 +2773,21 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Pepiniera Cobadin — Constanța</t>
+          <t>Pepiniera Selficom — Galați</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DN3, la intrarea în Cobadin · tel. 0746.037.827 · contact@pepinieracobadin.ro · lista de prețuri 2024–2025 primită la 6 octombrie (`raspunsuri/oferta-pepiniera-cobadin-2024-2025.md`) · 50 km de Crucea, se ridică personal</t>
+          <t>tel. 0765402805 · ofertă pe puietiforestieri.ro: sânger 1,2 lei, stejar pufos 1,5 lei, măceș 1 leu · același drum cu Matto Medusa</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lista lor de prețuri arată **material de amenajare, nu puieți de împădurire**: arbori de 3–9 ani și 1,5–3,5 m la 50–160 lei, arbuști de 0,5–1,5 m la 15–80 lei; sânger și tei argintiu nu sunt în listă. Pentru pădure rămâne de la ei doar cătina roșie (15 lei, 3 ani, peste 1,3 m, se scurtează la 50 cm la plantare). Arțarul tătăresc, scumpia și sâmbovina s-au mutat la Agigea, cu Mizil ca rezervă; sângerul la Selficom Galați. Cererea de ofertă trimisă rămâne valabilă: dacă au și mărimi mici din semănătură, cum au la salcâm japonez (5 lei), se revine.</t>
+          <t>Singura pepinieră din zonă cu sânger la preț silvic (Cobadin nu-l are în lista de prețuri). Se ridică odată cu stejarul pufos de la Matto Medusa, sau se cere Agigei.</t>
         </is>
       </c>
     </row>
@@ -2706,33 +2831,33 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Jf</t>
+          <t>Cs</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Cătină roșie (în locul iasomiei sălbatice)</t>
+          <t>Sânger</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Tamarix ramosissima</t>
+          <t>Cornus sanguinea</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>15,00 (2024)</t>
+          <t>1,20</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>strat D, manta; înlocuitor pentru iasomia sălbatică; alternativ planteieftine.ro Tamarix tetrandra, rădăcină liberă</t>
+          <t>strat C; alternativ Pepiniera Zăval (Dolj) 1,02 lei sau Agigea</t>
         </is>
       </c>
     </row>
@@ -2745,10 +2870,10 @@
       </c>
       <c r="C7" s="6" t="inlineStr"/>
       <c r="D7" s="6" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>

</xml_diff>